<commit_message>
research: update NMS literature map for October 2026
Add seven records with separate peer-reviewed and preprint evidence, correct CEINMS-RT journal status, and refresh taxonomy, screening, verification, gaps and workbook.
</commit_message>
<xml_diff>
--- a/01_literature_mapping/NMS_literature_map_first_pass.xlsx
+++ b/01_literature_mapping/NMS_literature_map_first_pass.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" r:id="Rdf84695a9817455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R11efd4d26beb4954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="3" r:id="Rbc3392e1d6aa4157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" r:id="R524c5f52b1c74bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9ed585ee33964dee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="3" r:id="R76dc31dcf1c84961"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,6 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
@@ -572,7 +575,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="265">
+  <x:cellXfs count="268">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1204,6 +1207,15 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1215,7 +1227,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -1225,7 +1237,7 @@
         <x:color rgb="FF783F04"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5CD"/>
         </x:patternFill>
       </x:fill>
@@ -1236,7 +1248,7 @@
         <x:color rgb="FF0B5394"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
@@ -1246,8 +1258,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LiteratureMatrixTable" displayName="LiteratureMatrixTable" ref="A1:R61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:R61"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LiteratureMatrixTable" displayName="LiteratureMatrixTable" ref="A1:R68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:R68"/>
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="year"/>
@@ -4791,24 +4803,24 @@
         <x:v>Early Yanan Sui rehabilitation link; complements later simulation-centric work.</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="48" customHeight="1">
+    <x:row r="60" ht="135" customHeight="1">
       <x:c r="A60" s="36" t="str">
         <x:v>ROB010</x:v>
       </x:c>
-      <x:c r="B60" s="36" t="str">
+      <x:c r="B60" s="36" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C60" s="34" t="str">
-        <x:v>Sartori et al.</x:v>
+        <x:v>Massimo Sartori; Mohamed I. Refai; Lucas Avanci Gaudio; Christopher P. Cop; Donatella Simonetti; Federica Damonte; Matthew Hambly; David G. Lloyd; Claudio Pizzolato; Guillaume Durandau</x:v>
       </x:c>
       <x:c r="D60" s="34" t="str">
-        <x:v>CEINMS-RT: an open-source framework for the continuous neuro-mechanical model-based control of wearable robots</x:v>
+        <x:v>CEINMS-RT: An Open-Source Framework for the Continuous Neuro-Mechanical Model-Based Control of Wearable Robots</x:v>
       </x:c>
       <x:c r="E60" s="34" t="str">
-        <x:v>TechRxiv</x:v>
+        <x:v>IEEE Transactions on Medical Robotics and Bionics</x:v>
       </x:c>
       <x:c r="F60" s="34" t="str">
-        <x:v>https://www.techrxiv.org/doi/full/10.36227/techrxiv.173808030.92454585</x:v>
+        <x:v>https://doi.org/10.1109/TMRB.2025.3643986</x:v>
       </x:c>
       <x:c r="G60" s="34" t="str">
         <x:v>Assistive robotics infrastructure</x:v>
@@ -4832,19 +4844,19 @@
         <x:v>assistive_control</x:v>
       </x:c>
       <x:c r="N60" s="34" t="str">
-        <x:v>Preprint/software demonstrations</x:v>
+        <x:v>Peer-reviewed software and real-time modeling evaluation</x:v>
       </x:c>
       <x:c r="O60" s="36" t="str">
         <x:v>twin_enabling</x:v>
       </x:c>
       <x:c r="P60" s="36" t="str">
-        <x:v>preprint_metadata_verified</x:v>
+        <x:v>metadata_and_abstract_verified</x:v>
       </x:c>
       <x:c r="Q60" s="36" t="str">
-        <x:v>watch</x:v>
+        <x:v>core</x:v>
       </x:c>
       <x:c r="R60" s="34" t="str">
-        <x:v>High strategic relevance; retain as preprint until peer-reviewed version is located.</x:v>
+        <x:v>Corrected 2026-10-01 from preprint to journal record. Early online 2025-12-15; issue 2026-03-09, 8(1):405-417. Year retains early-online convention (2025). Source: University of Twente publication record and IEEE DOI. Not a September-new study.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
@@ -4901,6 +4913,398 @@
       </x:c>
       <x:c r="R61" s="34" t="str">
         <x:v>Priority TRO clinical adaptation paper; biological NMS state is not fully explicit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="160" customHeight="1">
+      <x:c r="A62" s="266" t="str">
+        <x:v>NMS020</x:v>
+      </x:c>
+      <x:c r="B62" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C62" s="266" t="str">
+        <x:v>Alireza Y. Bavil; Ayda Karimi Dastgerdi; Rod S. Barrett; Bradley M. Cornish; Matthew J. Hambly; Matthew Carrall-Worsey; Claudio Pizzolato; Amir Esrafilian; Dale Robinson; Laurent Frossard; David John Saxby; Stefanie Feih; Christopher P. Carty; David G. Lloyd</x:v>
+      </x:c>
+      <x:c r="D62" s="266" t="str">
+        <x:v>Evidence-informed methodological approaches for coupled neuromusculoskeletal-finite element analysis workflows in orthopaedic biomechanics</x:v>
+      </x:c>
+      <x:c r="E62" s="266" t="str">
+        <x:v>Frontiers in Bioengineering and Biotechnology</x:v>
+      </x:c>
+      <x:c r="F62" s="266" t="str">
+        <x:v>https://doi.org/10.3389/fbioe.2026.1875782</x:v>
+      </x:c>
+      <x:c r="G62" s="266" t="str">
+        <x:v>Multiscale personalization</x:v>
+      </x:c>
+      <x:c r="H62" s="266" t="str">
+        <x:v>Orthopaedic surgical planning</x:v>
+      </x:c>
+      <x:c r="I62" s="266" t="str">
+        <x:v>Anatomy; movement; physiological loading</x:v>
+      </x:c>
+      <x:c r="J62" s="266" t="str">
+        <x:v>Coupled NMSK-FEA workflow recommendations and case exemplars</x:v>
+      </x:c>
+      <x:c r="K62" s="266" t="str">
+        <x:v>Patient geometry and loading</x:v>
+      </x:c>
+      <x:c r="L62" s="266" t="str">
+        <x:v>offline</x:v>
+      </x:c>
+      <x:c r="M62" s="266" t="str">
+        <x:v>Surgical decision-support methodology</x:v>
+      </x:c>
+      <x:c r="N62" s="266" t="str">
+        <x:v>Methods paper with ACL reconstruction and femoral osteotomy exemplars</x:v>
+      </x:c>
+      <x:c r="O62" s="266" t="str">
+        <x:v>twin_enabling</x:v>
+      </x:c>
+      <x:c r="P62" s="266" t="str">
+        <x:v>metadata_and_abstract_verified</x:v>
+      </x:c>
+      <x:c r="Q62" s="266" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="R62" s="266" t="str">
+        <x:v>Published 2026-09-03. Prospective outcome validation remains a future step; methodological guidance is not a validated longitudinal twin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="110" customHeight="1">
+      <x:c r="A63" s="266" t="str">
+        <x:v>NMS021</x:v>
+      </x:c>
+      <x:c r="B63" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C63" s="266" t="str">
+        <x:v>Yujia Gao; Shitan Wang; Yufeng Lin; Zilin Wang; Chenglong Feng; Lu Xiao; Chenghua Jiang; Wenxin Niu</x:v>
+      </x:c>
+      <x:c r="D63" s="266" t="str">
+        <x:v>Coupled Neuromusculoskeletal Finite Element Simulation Reveals Biomechanical Adaptation and Joint Tissue Risk of Ankle Exoskeleton Intervention after Stroke</x:v>
+      </x:c>
+      <x:c r="E63" s="266" t="str">
+        <x:v>Soft Robotics</x:v>
+      </x:c>
+      <x:c r="F63" s="266" t="str">
+        <x:v>https://doi.org/10.1177/21695172261486297</x:v>
+      </x:c>
+      <x:c r="G63" s="266" t="str">
+        <x:v>Multiscale personalization</x:v>
+      </x:c>
+      <x:c r="H63" s="266" t="str">
+        <x:v>Eight male chronic-stroke participants; two-week intervention</x:v>
+      </x:c>
+      <x:c r="I63" s="266" t="str">
+        <x:v>Pre/post biomechanical data</x:v>
+      </x:c>
+      <x:c r="J63" s="266" t="str">
+        <x:v>Synergy-informed NMS simulation coupled to personalized FE analysis</x:v>
+      </x:c>
+      <x:c r="K63" s="266" t="str">
+        <x:v>Personalized FE model</x:v>
+      </x:c>
+      <x:c r="L63" s="266" t="str">
+        <x:v>episodic</x:v>
+      </x:c>
+      <x:c r="M63" s="266" t="str">
+        <x:v>Offline assessment of exoskeleton intervention</x:v>
+      </x:c>
+      <x:c r="N63" s="266" t="str">
+        <x:v>Patient cohort plus model-derived internal loading</x:v>
+      </x:c>
+      <x:c r="O63" s="266" t="str">
+        <x:v>twin_enabling</x:v>
+      </x:c>
+      <x:c r="P63" s="266" t="str">
+        <x:v>metadata_and_abstract_verified</x:v>
+      </x:c>
+      <x:c r="Q63" s="266" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="R63" s="266" t="str">
+        <x:v>Published 2026-09-06. Predicted tissue loading is not direct evidence of degeneration. Abstract verified; full-text risk-of-bias and tissue validation pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="110" customHeight="1">
+      <x:c r="A64" s="266" t="str">
+        <x:v>ROB012</x:v>
+      </x:c>
+      <x:c r="B64" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C64" s="266" t="str">
+        <x:v>Tiago Coelho-Magalhães; Christine Azevedo-Coste; Henrique Resende-Martins; François Bailly</x:v>
+      </x:c>
+      <x:c r="D64" s="266" t="str">
+        <x:v>Personalized FES-cycling patterns via optimal control: from musculoskeletal simulation to experimental validation</x:v>
+      </x:c>
+      <x:c r="E64" s="266" t="str">
+        <x:v>Journal of NeuroEngineering and Rehabilitation</x:v>
+      </x:c>
+      <x:c r="F64" s="266" t="str">
+        <x:v>https://doi.org/10.1186/s12984-026-02136-x</x:v>
+      </x:c>
+      <x:c r="G64" s="266" t="str">
+        <x:v>Rehabilitation and assistive robotics</x:v>
+      </x:c>
+      <x:c r="H64" s="266" t="str">
+        <x:v>One participant with spinal cord injury</x:v>
+      </x:c>
+      <x:c r="I64" s="266" t="str">
+        <x:v>Evoked contraction calibration; cycling measurements</x:v>
+      </x:c>
+      <x:c r="J64" s="266" t="str">
+        <x:v>Physiological muscle model and trajectory optimization of stimulation pulse duration</x:v>
+      </x:c>
+      <x:c r="K64" s="266" t="str">
+        <x:v>Muscle parameters identified for participant</x:v>
+      </x:c>
+      <x:c r="L64" s="266" t="str">
+        <x:v>offline calibration</x:v>
+      </x:c>
+      <x:c r="M64" s="266" t="str">
+        <x:v>FES stimulation pattern</x:v>
+      </x:c>
+      <x:c r="N64" s="266" t="str">
+        <x:v>Single-participant experimental feasibility</x:v>
+      </x:c>
+      <x:c r="O64" s="266" t="str">
+        <x:v>twin_enabling</x:v>
+      </x:c>
+      <x:c r="P64" s="266" t="str">
+        <x:v>metadata_and_abstract_verified</x:v>
+      </x:c>
+      <x:c r="Q64" s="266" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="R64" s="266" t="str">
+        <x:v>Published 2026-09-04 as peer-reviewed accepted article. Patterns transferred to cycling without empirical modification; not longitudinal clinical efficacy or continuous twin updating.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="110" customHeight="1">
+      <x:c r="A65" s="266" t="str">
+        <x:v>NEU013</x:v>
+      </x:c>
+      <x:c r="B65" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C65" s="266" t="str">
+        <x:v>Gunwoo Park; Seungwoo Yoon; Friedl De Groote; Seungbum Koo</x:v>
+      </x:c>
+      <x:c r="D65" s="266" t="str">
+        <x:v>Spinal reflexes with dynamic gain modulation contribute to robust walking: a comparative study of simulated neural controllers</x:v>
+      </x:c>
+      <x:c r="E65" s="266" t="str">
+        <x:v>Journal of NeuroEngineering and Rehabilitation</x:v>
+      </x:c>
+      <x:c r="F65" s="266" t="str">
+        <x:v>https://doi.org/10.1186/s12984-026-02157-6</x:v>
+      </x:c>
+      <x:c r="G65" s="266" t="str">
+        <x:v>Neural control and embodied AI</x:v>
+      </x:c>
+      <x:c r="H65" s="266" t="str">
+        <x:v>Simulated human locomotion</x:v>
+      </x:c>
+      <x:c r="I65" s="266" t="str">
+        <x:v>Reference motion; simulated proprioceptive feedback</x:v>
+      </x:c>
+      <x:c r="J65" s="266" t="str">
+        <x:v>Virtual ablation of four neural architectures; PPO; 14-DOF 22-muscle model</x:v>
+      </x:c>
+      <x:c r="K65" s="266" t="str">
+        <x:v>No individual patient binding demonstrated</x:v>
+      </x:c>
+      <x:c r="L65" s="266" t="str">
+        <x:v>simulation</x:v>
+      </x:c>
+      <x:c r="M65" s="266" t="str">
+        <x:v>Simulated muscle excitation control</x:v>
+      </x:c>
+      <x:c r="N65" s="266" t="str">
+        <x:v>Simulation perturbation tests</x:v>
+      </x:c>
+      <x:c r="O65" s="266" t="str">
+        <x:v>simulation_only</x:v>
+      </x:c>
+      <x:c r="P65" s="266" t="str">
+        <x:v>metadata_and_abstract_verified</x:v>
+      </x:c>
+      <x:c r="Q65" s="266" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="R65" s="266" t="str">
+        <x:v>Published 2026-09-22 as peer-reviewed accepted article. Evidence for controller architecture in simulation, not direct proof of human neural mechanisms or patient safety.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="110" customHeight="1">
+      <x:c r="A66" s="266" t="str">
+        <x:v>ROB013</x:v>
+      </x:c>
+      <x:c r="B66" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C66" s="266" t="str">
+        <x:v>Yifei Yuan; Jakob Wolf; Ghaith Androwis; Xianlian Zhou</x:v>
+      </x:c>
+      <x:c r="D66" s="266" t="str">
+        <x:v>UniExo: Unified Multi-Skill Policies for Musculoskeletal Locomotion and Co-Adaptive Exoskeleton Control</x:v>
+      </x:c>
+      <x:c r="E66" s="266" t="str">
+        <x:v>arXiv preprint</x:v>
+      </x:c>
+      <x:c r="F66" s="266" t="str">
+        <x:v>https://arxiv.org/abs/2609.19690</x:v>
+      </x:c>
+      <x:c r="G66" s="266" t="str">
+        <x:v>Rehabilitation and assistive robotics</x:v>
+      </x:c>
+      <x:c r="H66" s="266" t="str">
+        <x:v>Six participants treadmill; one participant multi-skill route (abstract reports)</x:v>
+      </x:c>
+      <x:c r="I66" s="266" t="str">
+        <x:v>Imitation reference motion; device state</x:v>
+      </x:c>
+      <x:c r="J66" s="266" t="str">
+        <x:v>Expert distillation; multi-agent human/exoskeleton policy training</x:v>
+      </x:c>
+      <x:c r="K66" s="266" t="str">
+        <x:v>Individual NMS calibration not established by abstract</x:v>
+      </x:c>
+      <x:c r="L66" s="266" t="str">
+        <x:v>Device deployment; online patient model update not established</x:v>
+      </x:c>
+      <x:c r="M66" s="266" t="str">
+        <x:v>Hip-exoskeleton assistance</x:v>
+      </x:c>
+      <x:c r="N66" s="266" t="str">
+        <x:v>Simulation and reported human device demonstration</x:v>
+      </x:c>
+      <x:c r="O66" s="266" t="str">
+        <x:v>twin_enabling</x:v>
+      </x:c>
+      <x:c r="P66" s="266" t="str">
+        <x:v>preprint_metadata_verified</x:v>
+      </x:c>
+      <x:c r="Q66" s="266" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="R66" s="266" t="str">
+        <x:v>Submitted 2026-09-17. Indexed arXiv abstract inspected; direct page unavailable. Co-adaptation is training-stage; no patient recovery claim. Journal DOI and peer review unverified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="110" customHeight="1">
+      <x:c r="A67" s="266" t="str">
+        <x:v>EMB006</x:v>
+      </x:c>
+      <x:c r="B67" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C67" s="266" t="str">
+        <x:v>Mengtao Ou; Zongzheng Zhang; Zhenghao Xiao; Yixuan Pan; Ziwen Zhuang; Hang Zhao; Hongyang Li; Yanan Sui; Libin Liu; Hao Zhao</x:v>
+      </x:c>
+      <x:c r="D67" s="266" t="str">
+        <x:v>MSK-Bench: Benchmarking Full-Body Musculoskeletal Motor Control Across Tasks, Control Paradigms, and Physiological Metrics</x:v>
+      </x:c>
+      <x:c r="E67" s="266" t="str">
+        <x:v>arXiv preprint</x:v>
+      </x:c>
+      <x:c r="F67" s="266" t="str">
+        <x:v>https://arxiv.org/abs/2609.26872</x:v>
+      </x:c>
+      <x:c r="G67" s="266" t="str">
+        <x:v>Musculoskeletal embodied AI</x:v>
+      </x:c>
+      <x:c r="H67" s="266" t="str">
+        <x:v>Full-body simulated human; 22 tasks</x:v>
+      </x:c>
+      <x:c r="I67" s="266" t="str">
+        <x:v>Simulated state; motion and physiological reference metrics</x:v>
+      </x:c>
+      <x:c r="J67" s="266" t="str">
+        <x:v>Benchmark across task classes and control paradigms</x:v>
+      </x:c>
+      <x:c r="K67" s="266" t="str">
+        <x:v>No physical-person synchronization established</x:v>
+      </x:c>
+      <x:c r="L67" s="266" t="str">
+        <x:v>simulation</x:v>
+      </x:c>
+      <x:c r="M67" s="266" t="str">
+        <x:v>Simulated muscle-actuated control</x:v>
+      </x:c>
+      <x:c r="N67" s="266" t="str">
+        <x:v>Simulation benchmark; physiology-oriented diagnostics</x:v>
+      </x:c>
+      <x:c r="O67" s="266" t="str">
+        <x:v>simulation_only</x:v>
+      </x:c>
+      <x:c r="P67" s="266" t="str">
+        <x:v>preprint_metadata_verified</x:v>
+      </x:c>
+      <x:c r="Q67" s="266" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="R67" s="266" t="str">
+        <x:v>Submitted 2026-09-22. Indexed arXiv abstract inspected; direct page unavailable. EMG similarity does not identify unique neural control. Journal DOI and conference acceptance unverified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="110" customHeight="1">
+      <x:c r="A68" s="266" t="str">
+        <x:v>WEA008</x:v>
+      </x:c>
+      <x:c r="B68" s="266" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C68" s="266" t="str">
+        <x:v>Erica L. King; Connor Delaney; Morgan A. Lamarre; Amad Qureshi; Siddhartha Sikdar; Qi Wei; Parag V. Chitnis</x:v>
+      </x:c>
+      <x:c r="D68" s="266" t="str">
+        <x:v>Comparative Analysis of Muscle Fascia Tracking Algorithms for Real-Time Muscle Monitoring using Wearable Ultrasound</x:v>
+      </x:c>
+      <x:c r="E68" s="266" t="str">
+        <x:v>IEEE Journal of Biomedical and Health Informatics</x:v>
+      </x:c>
+      <x:c r="F68" s="266" t="str">
+        <x:v>https://doi.org/10.1109/JBHI.2026.3734932</x:v>
+      </x:c>
+      <x:c r="G68" s="266" t="str">
+        <x:v>Wearable observability</x:v>
+      </x:c>
+      <x:c r="H68" s="266" t="str">
+        <x:v>Quadriceps isometric activation and squats; 572 images</x:v>
+      </x:c>
+      <x:c r="I68" s="266" t="str">
+        <x:v>Multi-site M-mode wearable ultrasound</x:v>
+      </x:c>
+      <x:c r="J68" s="266" t="str">
+        <x:v>Five fascia-tracking methods compared to expert annotations</x:v>
+      </x:c>
+      <x:c r="K68" s="266" t="str">
+        <x:v>No NMS parameter calibration demonstrated</x:v>
+      </x:c>
+      <x:c r="L68" s="266" t="str">
+        <x:v>Wearable monitoring context</x:v>
+      </x:c>
+      <x:c r="M68" s="266" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="N68" s="266" t="str">
+        <x:v>Image-level fascia tracking validation</x:v>
+      </x:c>
+      <x:c r="O68" s="266" t="str">
+        <x:v>twin_enabling</x:v>
+      </x:c>
+      <x:c r="P68" s="266" t="str">
+        <x:v>metadata_and_abstract_verified</x:v>
+      </x:c>
+      <x:c r="Q68" s="266" t="str">
+        <x:v>adjacent</x:v>
+      </x:c>
+      <x:c r="R68" s="266" t="str">
+        <x:v>Journal online 2026-09-16; July medRxiv predecessor is the same study, not another record. Image count is not participant count; fascia displacement is not muscle force truth.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4921,7 +5325,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fc0b1b786f44f86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R888e1ab64b944450"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4940,9 +5344,9 @@
     <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="38" customHeight="1">
+    <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="164" t="str">
-        <x:v>Human Neuromusculoskeletal Digital Twin / Embodied AI — First-Pass Map</x:v>
+        <x:v>Human Neuromusculoskeletal Digital Twin / Embodied AI — Updated Map</x:v>
       </x:c>
       <x:c r="B1" s="164"/>
       <x:c r="C1" s="164"/>
@@ -4966,28 +5370,28 @@
       <x:c r="A3" s="166" t="str">
         <x:v>Search cutoff</x:v>
       </x:c>
-      <x:c r="B3" s="167" t="str">
-        <x:v>2026-09-01</x:v>
+      <x:c r="B3" s="267" t="n">
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C3" s="168" t="str">
         <x:v>Mapped papers</x:v>
       </x:c>
       <x:c r="D3" s="168" t="n">
-        <x:f>COUNTA('Literature Matrix'!$A$2:$A$61)</x:f>
-        <x:v>60</x:v>
+        <x:f>COUNTA('Literature Matrix'!$A$2:$A$68)</x:f>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="E3" s="168" t="str">
         <x:v>Core papers</x:v>
       </x:c>
       <x:c r="F3" s="168" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$Q$2:$Q$61,"core")</x:f>
-        <x:v>49</x:v>
+        <x:f>COUNTIF('Literature Matrix'!$Q$2:$Q$68,"core")</x:f>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="G3" s="168" t="str">
         <x:v>Explicit DT</x:v>
       </x:c>
       <x:c r="H3" s="169" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$61,"explicit_digital_twin")</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$68,"explicit_digital_twin")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -5036,7 +5440,7 @@
         <x:v>explicit_digital_twin</x:v>
       </x:c>
       <x:c r="E6" s="174" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$61,D6)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$68,D6)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F6" s="165"/>
@@ -5044,7 +5448,7 @@
         <x:v>IEEE Transactions on Neural Systems and Rehabilitation Engineering</x:v>
       </x:c>
       <x:c r="H6" s="174" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G6)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G6)</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -5053,23 +5457,23 @@
         <x:v>NMS/personalization</x:v>
       </x:c>
       <x:c r="B7" s="176" t="n">
-        <x:f>COUNTA('Literature Matrix'!$A$8:$A$26)</x:f>
-        <x:v>19</x:v>
+        <x:f>COUNTA('Literature Matrix'!$A$8:$A$26,'Literature Matrix'!$A$62:$A$63)</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C7" s="165"/>
       <x:c r="D7" s="175" t="str">
         <x:v>twin_enabling</x:v>
       </x:c>
       <x:c r="E7" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$61,D7)</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$68,D7)</x:f>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F7" s="165"/>
       <x:c r="G7" s="175" t="str">
         <x:v>IEEE Transactions on Biomedical Engineering</x:v>
       </x:c>
       <x:c r="H7" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G7)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G7)</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -5078,24 +5482,24 @@
         <x:v>Neural control</x:v>
       </x:c>
       <x:c r="B8" s="176" t="n">
-        <x:f>COUNTA('Literature Matrix'!$A$27:$A$38)</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTA('Literature Matrix'!$A$27:$A$38,'Literature Matrix'!$A$65)</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C8" s="165"/>
       <x:c r="D8" s="175" t="str">
         <x:v>simulation_only</x:v>
       </x:c>
       <x:c r="E8" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$61,D8)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$68,D8)</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F8" s="165"/>
       <x:c r="G8" s="175" t="str">
         <x:v>IEEE Journal of Biomedical and Health Informatics</x:v>
       </x:c>
       <x:c r="H8" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G8)</x:f>
-        <x:v>3</x:v>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G8)</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5103,15 +5507,15 @@
         <x:v>Embodied AI</x:v>
       </x:c>
       <x:c r="B9" s="176" t="n">
-        <x:f>COUNTA('Literature Matrix'!$A$39:$A$43)</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTA('Literature Matrix'!$A$39:$A$43,'Literature Matrix'!$A$67)</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C9" s="165"/>
       <x:c r="D9" s="178" t="str">
         <x:v>review</x:v>
       </x:c>
       <x:c r="E9" s="179" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$61,D9)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$O$2:$O$68,D9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F9" s="165"/>
@@ -5119,7 +5523,7 @@
         <x:v>IEEE Transactions on Robotics</x:v>
       </x:c>
       <x:c r="H9" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G9)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G9)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -5128,8 +5532,8 @@
         <x:v>Wearable observability</x:v>
       </x:c>
       <x:c r="B10" s="176" t="n">
-        <x:f>COUNTA('Literature Matrix'!$A$44:$A$50)</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTA('Literature Matrix'!$A$44:$A$50,'Literature Matrix'!$A$68)</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="165"/>
       <x:c r="D10" s="165"/>
@@ -5139,7 +5543,7 @@
         <x:v>Scientific Reports</x:v>
       </x:c>
       <x:c r="H10" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G10)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G10)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -5148,8 +5552,8 @@
         <x:v>Rehabilitation/robotics</x:v>
       </x:c>
       <x:c r="B11" s="180" t="n">
-        <x:f>COUNTA('Literature Matrix'!$A$51:$A$61)</x:f>
-        <x:v>11</x:v>
+        <x:f>COUNTA('Literature Matrix'!$A$51:$A$61,'Literature Matrix'!$A$64,'Literature Matrix'!$A$66)</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C11" s="165"/>
       <x:c r="D11" s="165"/>
@@ -5159,8 +5563,8 @@
         <x:v>Journal of NeuroEngineering and Rehabilitation</x:v>
       </x:c>
       <x:c r="H11" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G11)</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G11)</x:f>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5174,7 +5578,7 @@
         <x:v>Journal of Biomechanics</x:v>
       </x:c>
       <x:c r="H12" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G12)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G12)</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -5189,7 +5593,7 @@
         <x:v>NeurIPS</x:v>
       </x:c>
       <x:c r="H13" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G13)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G13)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -5204,7 +5608,7 @@
         <x:v>ICML</x:v>
       </x:c>
       <x:c r="H14" s="177" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G14)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G14)</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -5219,7 +5623,7 @@
         <x:v>ICRA</x:v>
       </x:c>
       <x:c r="H15" s="179" t="n">
-        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$61,G15)</x:f>
+        <x:f>COUNTIF('Literature Matrix'!$E$2:$E$68,G15)</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -5233,9 +5637,9 @@
       <x:c r="G16" s="165"/>
       <x:c r="H16" s="165"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="181" t="str">
-        <x:v>Interpretation: most records are twin-enabling components. Embodied AI papers usually provide scalable simulated control, while the strongest patient-facing closed loops are real-time NMS-driven prosthesis/exoskeleton interfaces. A synchronized, uncertainty-aware, longitudinal L5 patient twin was not identified in this seed set.</x:v>
+        <x:v>Update 2026-10-01: 7 additions (5 journal articles, 2 preprint watch items), 1 publication-status correction, 0 deletions. New evidence links tissue modeling, neural control, FES, wearable ultrasound and multi-skill assistance. No complete longitudinal patient twin verified. See dated search and screening logs.</x:v>
       </x:c>
       <x:c r="B17" s="182"/>
       <x:c r="C17" s="182"/>
@@ -5245,7 +5649,7 @@
       <x:c r="G17" s="182"/>
       <x:c r="H17" s="183"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="184"/>
       <x:c r="B18" s="185"/>
       <x:c r="C18" s="185"/>
@@ -5255,7 +5659,7 @@
       <x:c r="G18" s="185"/>
       <x:c r="H18" s="186"/>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="187"/>
       <x:c r="B19" s="188"/>
       <x:c r="C19" s="188"/>
@@ -5315,7 +5719,7 @@
         <x:v>Stable seed-map identifier and research-stream prefix.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="44" customHeight="1">
+    <x:row r="3" ht="65" customHeight="1">
       <x:c r="A3" s="259" t="str">
         <x:v>year</x:v>
       </x:c>
@@ -5323,7 +5727,7 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="C3" s="261" t="str">
-        <x:v>Publication year; online-ahead-of-print year used when applicable.</x:v>
+        <x:v>Earliest verified journal online year when known; issue date and preprint history recorded separately in dated verification CSV.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="44" customHeight="1">
@@ -5469,7 +5873,7 @@
         <x:v>Evidence-aware relationship to digital-twin concept.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="44" customHeight="1">
+    <x:row r="17" ht="65" customHeight="1">
       <x:c r="A17" s="259" t="str">
         <x:v>evidence_status</x:v>
       </x:c>
@@ -5477,7 +5881,7 @@
         <x:v>metadata_verified / metadata_and_abstract_verified / full_text_sections_verified / preprint_metadata_verified</x:v>
       </x:c>
       <x:c r="C17" s="261" t="str">
-        <x:v>Depth of source inspection in round one.</x:v>
+        <x:v>Depth of actual source inspection. Preprint watch items remain separate; indexed-abstract-only access is stated in screening notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="44" customHeight="1">

</xml_diff>